<commit_message>
Ajout des exemples manquants, restriction du appointement sur le FRpractionner au lieu de Practitionner et lien avec FrCorePatientProfile au lieu de FrCorePatientINSProfile a4489a6b0d7c45749cba290f5d7ea5e1c23d78d6
</commit_message>
<xml_diff>
--- a/nmoreau/ig/StructureDefinition-preadmission-appointment-fr.xlsx
+++ b/nmoreau/ig/StructureDefinition-preadmission-appointment-fr.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-04-25T14:29:23+00:00</t>
+    <t>2025-04-25T16:50:14+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1216,7 +1216,7 @@
     <t>Appointment.participant.actor</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-patient-ins)
+    <t xml:space="preserve">Reference(https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-patient|https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-patient)
 </t>
   </si>
   <si>
@@ -1635,7 +1635,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="100.99609375" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="103.15625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>

</xml_diff>

<commit_message>
#16 : ajout de https://smt.esante.gouv.fr/fhir/ValueSet/JDV-J66-TypeCode-DMP à la valueset des types de documents possibles 69c8df34255daf56dfd69531f59cc2e17be36582
</commit_message>
<xml_diff>
--- a/nmoreau/ig/StructureDefinition-preadmission-appointment-fr.xlsx
+++ b/nmoreau/ig/StructureDefinition-preadmission-appointment-fr.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1902" uniqueCount="411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1865" uniqueCount="406">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-01-14T12:51:21+00:00</t>
+    <t>2026-02-24T09:27:09+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -648,22 +648,6 @@
   <si>
     <t xml:space="preserve">ele-1
 </t>
-  </si>
-  <si>
-    <t>Appointment.extension:questionnaire</t>
-  </si>
-  <si>
-    <t>questionnaire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extension {http://hl7.fr/fhir/fr/preadmission/StructureDefinition/appointment-questionnaire-response}
-</t>
-  </si>
-  <si>
-    <t>Questionnaire lié au rendez-vous</t>
-  </si>
-  <si>
-    <t>Référence vers un ou plusieurs QuestionnaireResponse remplis dans le cadre de la préadmission.</t>
   </si>
   <si>
     <t>Appointment.modifierExtension</t>
@@ -1606,7 +1590,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AO51"/>
+  <dimension ref="A1:AO50"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="36.921875" customWidth="true" bestFit="true"/>
@@ -3879,13 +3863,11 @@
         <v>204</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>194</v>
-      </c>
-      <c r="C20" t="s" s="2">
-        <v>205</v>
-      </c>
+        <v>204</v>
+      </c>
+      <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
-        <v>79</v>
+        <v>110</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" t="s" s="2">
@@ -3898,22 +3880,26 @@
         <v>79</v>
       </c>
       <c r="I20" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="J20" t="s" s="2">
         <v>79</v>
       </c>
       <c r="K20" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L20" t="s" s="2">
+        <v>205</v>
+      </c>
+      <c r="M20" t="s" s="2">
         <v>206</v>
       </c>
-      <c r="L20" t="s" s="2">
+      <c r="N20" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="O20" t="s" s="2">
         <v>207</v>
       </c>
-      <c r="M20" t="s" s="2">
-        <v>208</v>
-      </c>
-      <c r="N20" s="2"/>
-      <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
         <v>79</v>
       </c>
@@ -3961,7 +3947,7 @@
         <v>79</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>80</v>
@@ -3979,7 +3965,7 @@
         <v>79</v>
       </c>
       <c r="AL20" t="s" s="2">
-        <v>79</v>
+        <v>193</v>
       </c>
       <c r="AM20" t="s" s="2">
         <v>79</v>
@@ -4000,7 +3986,7 @@
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="E21" s="2"/>
       <c r="F21" t="s" s="2">
@@ -4013,26 +3999,22 @@
         <v>79</v>
       </c>
       <c r="I21" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="J21" t="s" s="2">
         <v>91</v>
       </c>
-      <c r="J21" t="s" s="2">
-        <v>79</v>
-      </c>
       <c r="K21" t="s" s="2">
-        <v>111</v>
+        <v>210</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>211</v>
-      </c>
-      <c r="N21" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="O21" t="s" s="2">
         <v>212</v>
       </c>
+      <c r="N21" s="2"/>
+      <c r="O21" s="2"/>
       <c r="P21" t="s" s="2">
         <v>79</v>
       </c>
@@ -4080,7 +4062,7 @@
         <v>79</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>80</v>
@@ -4092,30 +4074,30 @@
         <v>79</v>
       </c>
       <c r="AJ21" t="s" s="2">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="AK21" t="s" s="2">
-        <v>79</v>
+        <v>213</v>
       </c>
       <c r="AL21" t="s" s="2">
-        <v>193</v>
+        <v>214</v>
       </c>
       <c r="AM21" t="s" s="2">
-        <v>79</v>
+        <v>215</v>
       </c>
       <c r="AN21" t="s" s="2">
-        <v>79</v>
+        <v>216</v>
       </c>
       <c r="AO21" t="s" s="2">
-        <v>79</v>
+        <v>217</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -4123,30 +4105,32 @@
       </c>
       <c r="E22" s="2"/>
       <c r="F22" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G22" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H22" t="s" s="2">
         <v>79</v>
       </c>
       <c r="I22" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="J22" t="s" s="2">
         <v>91</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>215</v>
+        <v>170</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>217</v>
-      </c>
-      <c r="N22" s="2"/>
+        <v>220</v>
+      </c>
+      <c r="N22" t="s" s="2">
+        <v>221</v>
+      </c>
       <c r="O22" s="2"/>
       <c r="P22" t="s" s="2">
         <v>79</v>
@@ -4171,13 +4155,13 @@
         <v>79</v>
       </c>
       <c r="X22" t="s" s="2">
-        <v>79</v>
+        <v>222</v>
       </c>
       <c r="Y22" t="s" s="2">
-        <v>79</v>
+        <v>223</v>
       </c>
       <c r="Z22" t="s" s="2">
-        <v>79</v>
+        <v>224</v>
       </c>
       <c r="AA22" t="s" s="2">
         <v>79</v>
@@ -4195,13 +4179,13 @@
         <v>79</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="AG22" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="AH22" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="AI22" t="s" s="2">
         <v>79</v>
@@ -4210,27 +4194,27 @@
         <v>102</v>
       </c>
       <c r="AK22" t="s" s="2">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="AL22" t="s" s="2">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="AM22" t="s" s="2">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="AN22" t="s" s="2">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="AO22" t="s" s="2">
-        <v>222</v>
+        <v>229</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -4238,7 +4222,7 @@
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G23" t="s" s="2">
         <v>90</v>
@@ -4247,23 +4231,21 @@
         <v>79</v>
       </c>
       <c r="I23" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="J23" t="s" s="2">
         <v>91</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>170</v>
+        <v>231</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>225</v>
-      </c>
-      <c r="N23" t="s" s="2">
-        <v>226</v>
-      </c>
+        <v>233</v>
+      </c>
+      <c r="N23" s="2"/>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
         <v>79</v>
@@ -4288,13 +4270,11 @@
         <v>79</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>227</v>
-      </c>
-      <c r="Y23" t="s" s="2">
-        <v>228</v>
-      </c>
+        <v>160</v>
+      </c>
+      <c r="Y23" s="2"/>
       <c r="Z23" t="s" s="2">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>79</v>
@@ -4312,10 +4292,10 @@
         <v>79</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="AG23" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="AH23" t="s" s="2">
         <v>90</v>
@@ -4327,19 +4307,19 @@
         <v>102</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>230</v>
+        <v>79</v>
       </c>
       <c r="AL23" t="s" s="2">
-        <v>231</v>
+        <v>108</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>232</v>
+        <v>79</v>
       </c>
       <c r="AN23" t="s" s="2">
-        <v>233</v>
+        <v>79</v>
       </c>
       <c r="AO23" t="s" s="2">
-        <v>234</v>
+        <v>79</v>
       </c>
     </row>
     <row r="24">
@@ -4358,7 +4338,7 @@
         <v>80</v>
       </c>
       <c r="G24" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="H24" t="s" s="2">
         <v>79</v>
@@ -4370,13 +4350,13 @@
         <v>91</v>
       </c>
       <c r="K24" t="s" s="2">
+        <v>231</v>
+      </c>
+      <c r="L24" t="s" s="2">
         <v>236</v>
       </c>
-      <c r="L24" t="s" s="2">
+      <c r="M24" t="s" s="2">
         <v>237</v>
-      </c>
-      <c r="M24" t="s" s="2">
-        <v>238</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -4407,7 +4387,7 @@
       </c>
       <c r="Y24" s="2"/>
       <c r="Z24" t="s" s="2">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="AA24" t="s" s="2">
         <v>79</v>
@@ -4431,7 +4411,7 @@
         <v>80</v>
       </c>
       <c r="AH24" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI24" t="s" s="2">
         <v>79</v>
@@ -4443,10 +4423,10 @@
         <v>79</v>
       </c>
       <c r="AL24" t="s" s="2">
-        <v>108</v>
+        <v>239</v>
       </c>
       <c r="AM24" t="s" s="2">
-        <v>79</v>
+        <v>240</v>
       </c>
       <c r="AN24" t="s" s="2">
         <v>79</v>
@@ -4457,10 +4437,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4483,15 +4463,17 @@
         <v>91</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>242</v>
-      </c>
-      <c r="N25" s="2"/>
+        <v>243</v>
+      </c>
+      <c r="N25" t="s" s="2">
+        <v>244</v>
+      </c>
       <c r="O25" s="2"/>
       <c r="P25" t="s" s="2">
         <v>79</v>
@@ -4520,7 +4502,7 @@
       </c>
       <c r="Y25" s="2"/>
       <c r="Z25" t="s" s="2">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="AA25" t="s" s="2">
         <v>79</v>
@@ -4538,7 +4520,7 @@
         <v>79</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>80</v>
@@ -4553,13 +4535,13 @@
         <v>102</v>
       </c>
       <c r="AK25" t="s" s="2">
-        <v>79</v>
+        <v>246</v>
       </c>
       <c r="AL25" t="s" s="2">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="AM25" t="s" s="2">
-        <v>245</v>
+        <v>79</v>
       </c>
       <c r="AN25" t="s" s="2">
         <v>79</v>
@@ -4570,10 +4552,10 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4596,17 +4578,15 @@
         <v>91</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>248</v>
-      </c>
-      <c r="N26" t="s" s="2">
         <v>249</v>
       </c>
+      <c r="N26" s="2"/>
       <c r="O26" s="2"/>
       <c r="P26" t="s" s="2">
         <v>79</v>
@@ -4631,7 +4611,7 @@
         <v>79</v>
       </c>
       <c r="X26" t="s" s="2">
-        <v>160</v>
+        <v>222</v>
       </c>
       <c r="Y26" s="2"/>
       <c r="Z26" t="s" s="2">
@@ -4653,7 +4633,7 @@
         <v>79</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>80</v>
@@ -4668,16 +4648,16 @@
         <v>102</v>
       </c>
       <c r="AK26" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AL26" t="s" s="2">
         <v>251</v>
       </c>
-      <c r="AL26" t="s" s="2">
-        <v>244</v>
-      </c>
       <c r="AM26" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AN26" t="s" s="2">
-        <v>79</v>
+        <v>252</v>
       </c>
       <c r="AO26" t="s" s="2">
         <v>79</v>
@@ -4685,10 +4665,10 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4699,7 +4679,7 @@
         <v>80</v>
       </c>
       <c r="G27" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H27" t="s" s="2">
         <v>79</v>
@@ -4711,13 +4691,13 @@
         <v>91</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -4744,11 +4724,11 @@
         <v>79</v>
       </c>
       <c r="X27" t="s" s="2">
-        <v>227</v>
+        <v>174</v>
       </c>
       <c r="Y27" s="2"/>
       <c r="Z27" t="s" s="2">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AA27" t="s" s="2">
         <v>79</v>
@@ -4766,13 +4746,13 @@
         <v>79</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH27" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="AI27" t="s" s="2">
         <v>79</v>
@@ -4784,24 +4764,24 @@
         <v>79</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="AM27" t="s" s="2">
-        <v>79</v>
+        <v>258</v>
       </c>
       <c r="AN27" t="s" s="2">
-        <v>257</v>
+        <v>79</v>
       </c>
       <c r="AO27" t="s" s="2">
-        <v>79</v>
+        <v>259</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4812,7 +4792,7 @@
         <v>80</v>
       </c>
       <c r="G28" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="H28" t="s" s="2">
         <v>79</v>
@@ -4824,13 +4804,13 @@
         <v>91</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -4859,9 +4839,11 @@
       <c r="X28" t="s" s="2">
         <v>174</v>
       </c>
-      <c r="Y28" s="2"/>
+      <c r="Y28" t="s" s="2">
+        <v>263</v>
+      </c>
       <c r="Z28" t="s" s="2">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="AA28" t="s" s="2">
         <v>79</v>
@@ -4879,13 +4861,13 @@
         <v>79</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH28" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI28" t="s" s="2">
         <v>79</v>
@@ -4894,27 +4876,27 @@
         <v>102</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>79</v>
+        <v>265</v>
       </c>
       <c r="AL28" t="s" s="2">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="AM28" t="s" s="2">
-        <v>263</v>
+        <v>79</v>
       </c>
       <c r="AN28" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AO28" t="s" s="2">
-        <v>264</v>
+        <v>267</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4934,16 +4916,16 @@
         <v>79</v>
       </c>
       <c r="J29" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>236</v>
+        <v>269</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
@@ -4970,31 +4952,31 @@
         <v>79</v>
       </c>
       <c r="X29" t="s" s="2">
-        <v>174</v>
+        <v>79</v>
       </c>
       <c r="Y29" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Z29" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AA29" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AB29" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AC29" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD29" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE29" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF29" t="s" s="2">
         <v>268</v>
-      </c>
-      <c r="Z29" t="s" s="2">
-        <v>269</v>
-      </c>
-      <c r="AA29" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB29" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC29" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD29" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE29" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF29" t="s" s="2">
-        <v>265</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>80</v>
@@ -5009,10 +4991,10 @@
         <v>102</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="AL29" t="s" s="2">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="AM29" t="s" s="2">
         <v>79</v>
@@ -5021,15 +5003,15 @@
         <v>79</v>
       </c>
       <c r="AO29" t="s" s="2">
-        <v>272</v>
+        <v>79</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -5040,7 +5022,7 @@
         <v>80</v>
       </c>
       <c r="G30" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H30" t="s" s="2">
         <v>79</v>
@@ -5052,15 +5034,17 @@
         <v>79</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>276</v>
-      </c>
-      <c r="N30" s="2"/>
+        <v>277</v>
+      </c>
+      <c r="N30" t="s" s="2">
+        <v>278</v>
+      </c>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
         <v>79</v>
@@ -5109,13 +5093,13 @@
         <v>79</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH30" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="AI30" t="s" s="2">
         <v>79</v>
@@ -5124,27 +5108,27 @@
         <v>102</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="AM30" t="s" s="2">
-        <v>79</v>
+        <v>281</v>
       </c>
       <c r="AN30" t="s" s="2">
-        <v>79</v>
+        <v>252</v>
       </c>
       <c r="AO30" t="s" s="2">
-        <v>79</v>
+        <v>282</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -5167,17 +5151,15 @@
         <v>79</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>280</v>
+        <v>104</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>282</v>
-      </c>
-      <c r="N31" t="s" s="2">
-        <v>283</v>
-      </c>
+        <v>285</v>
+      </c>
+      <c r="N31" s="2"/>
       <c r="O31" s="2"/>
       <c r="P31" t="s" s="2">
         <v>79</v>
@@ -5226,7 +5208,7 @@
         <v>79</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>80</v>
@@ -5241,27 +5223,27 @@
         <v>102</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>284</v>
+        <v>79</v>
       </c>
       <c r="AL31" t="s" s="2">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="AM31" t="s" s="2">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="AN31" t="s" s="2">
-        <v>257</v>
+        <v>79</v>
       </c>
       <c r="AO31" t="s" s="2">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -5272,7 +5254,7 @@
         <v>80</v>
       </c>
       <c r="G32" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="H32" t="s" s="2">
         <v>79</v>
@@ -5284,13 +5266,13 @@
         <v>79</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>104</v>
+        <v>290</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -5341,13 +5323,13 @@
         <v>79</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH32" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI32" t="s" s="2">
         <v>79</v>
@@ -5356,27 +5338,27 @@
         <v>102</v>
       </c>
       <c r="AK32" t="s" s="2">
-        <v>79</v>
+        <v>293</v>
       </c>
       <c r="AL32" t="s" s="2">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="AM32" t="s" s="2">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="AN32" t="s" s="2">
-        <v>79</v>
+        <v>296</v>
       </c>
       <c r="AO32" t="s" s="2">
-        <v>293</v>
+        <v>79</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5387,7 +5369,7 @@
         <v>80</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H33" t="s" s="2">
         <v>79</v>
@@ -5396,16 +5378,16 @@
         <v>79</v>
       </c>
       <c r="J33" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>295</v>
+        <v>126</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
@@ -5456,13 +5438,13 @@
         <v>79</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH33" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="AI33" t="s" s="2">
         <v>79</v>
@@ -5471,27 +5453,27 @@
         <v>102</v>
       </c>
       <c r="AK33" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL33" t="s" s="2">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="AM33" t="s" s="2">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="AN33" t="s" s="2">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="AO33" t="s" s="2">
-        <v>79</v>
+        <v>304</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5517,10 +5499,10 @@
         <v>126</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -5571,7 +5553,7 @@
         <v>79</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>80</v>
@@ -5586,27 +5568,27 @@
         <v>102</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="AL34" t="s" s="2">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="AM34" t="s" s="2">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="AN34" t="s" s="2">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="AO34" t="s" s="2">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5626,16 +5608,16 @@
         <v>79</v>
       </c>
       <c r="J35" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>126</v>
+        <v>313</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
@@ -5686,7 +5668,7 @@
         <v>79</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>80</v>
@@ -5701,27 +5683,27 @@
         <v>102</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="AL35" t="s" s="2">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="AM35" t="s" s="2">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="AN35" t="s" s="2">
-        <v>315</v>
+        <v>79</v>
       </c>
       <c r="AO35" t="s" s="2">
-        <v>316</v>
+        <v>79</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5732,7 +5714,7 @@
         <v>80</v>
       </c>
       <c r="G36" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="H36" t="s" s="2">
         <v>79</v>
@@ -5744,13 +5726,13 @@
         <v>79</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -5801,13 +5783,13 @@
         <v>79</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH36" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI36" t="s" s="2">
         <v>79</v>
@@ -5816,13 +5798,13 @@
         <v>102</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>305</v>
+        <v>79</v>
       </c>
       <c r="AL36" t="s" s="2">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="AM36" t="s" s="2">
-        <v>322</v>
+        <v>79</v>
       </c>
       <c r="AN36" t="s" s="2">
         <v>79</v>
@@ -5847,7 +5829,7 @@
         <v>80</v>
       </c>
       <c r="G37" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H37" t="s" s="2">
         <v>79</v>
@@ -5867,7 +5849,9 @@
       <c r="M37" t="s" s="2">
         <v>326</v>
       </c>
-      <c r="N37" s="2"/>
+      <c r="N37" t="s" s="2">
+        <v>327</v>
+      </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
         <v>79</v>
@@ -5922,7 +5906,7 @@
         <v>80</v>
       </c>
       <c r="AH37" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="AI37" t="s" s="2">
         <v>79</v>
@@ -5931,13 +5915,13 @@
         <v>102</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>79</v>
+        <v>328</v>
       </c>
       <c r="AL37" t="s" s="2">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="AM37" t="s" s="2">
-        <v>79</v>
+        <v>330</v>
       </c>
       <c r="AN37" t="s" s="2">
         <v>79</v>
@@ -5948,10 +5932,10 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5974,16 +5958,16 @@
         <v>79</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>329</v>
+        <v>104</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="N38" t="s" s="2">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
@@ -6033,7 +6017,7 @@
         <v>79</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>80</v>
@@ -6048,27 +6032,27 @@
         <v>102</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="AL38" t="s" s="2">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="AN38" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AO38" t="s" s="2">
-        <v>79</v>
+        <v>288</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -6094,14 +6078,12 @@
         <v>104</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>338</v>
-      </c>
-      <c r="N39" t="s" s="2">
-        <v>339</v>
-      </c>
+        <v>340</v>
+      </c>
+      <c r="N39" s="2"/>
       <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
         <v>79</v>
@@ -6150,7 +6132,7 @@
         <v>79</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>80</v>
@@ -6165,38 +6147,38 @@
         <v>102</v>
       </c>
       <c r="AK39" t="s" s="2">
-        <v>340</v>
+        <v>79</v>
       </c>
       <c r="AL39" t="s" s="2">
+        <v>336</v>
+      </c>
+      <c r="AM39" t="s" s="2">
         <v>341</v>
       </c>
-      <c r="AM39" t="s" s="2">
-        <v>342</v>
-      </c>
       <c r="AN39" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AO39" t="s" s="2">
-        <v>293</v>
+        <v>288</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
-        <v>79</v>
+        <v>343</v>
       </c>
       <c r="E40" s="2"/>
       <c r="F40" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G40" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="H40" t="s" s="2">
         <v>79</v>
@@ -6208,13 +6190,13 @@
         <v>79</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>104</v>
+        <v>344</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -6265,13 +6247,13 @@
         <v>79</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH40" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI40" t="s" s="2">
         <v>79</v>
@@ -6280,35 +6262,35 @@
         <v>102</v>
       </c>
       <c r="AK40" t="s" s="2">
-        <v>79</v>
+        <v>347</v>
       </c>
       <c r="AL40" t="s" s="2">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="AM40" t="s" s="2">
-        <v>346</v>
+        <v>79</v>
       </c>
       <c r="AN40" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AO40" t="s" s="2">
-        <v>293</v>
+        <v>79</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
-        <v>348</v>
+        <v>79</v>
       </c>
       <c r="E41" s="2"/>
       <c r="F41" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G41" t="s" s="2">
         <v>81</v>
@@ -6323,13 +6305,13 @@
         <v>79</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -6380,10 +6362,10 @@
         <v>79</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="AG41" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="AH41" t="s" s="2">
         <v>81</v>
@@ -6392,30 +6374,30 @@
         <v>79</v>
       </c>
       <c r="AJ41" t="s" s="2">
-        <v>102</v>
+        <v>353</v>
       </c>
       <c r="AK41" t="s" s="2">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="AL41" t="s" s="2">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="AM41" t="s" s="2">
-        <v>79</v>
+        <v>356</v>
       </c>
       <c r="AN41" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AO41" t="s" s="2">
-        <v>79</v>
+        <v>357</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6423,11 +6405,11 @@
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G42" t="s" s="2">
         <v>90</v>
       </c>
-      <c r="G42" t="s" s="2">
-        <v>81</v>
-      </c>
       <c r="H42" t="s" s="2">
         <v>79</v>
       </c>
@@ -6438,13 +6420,13 @@
         <v>79</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>355</v>
+        <v>104</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>356</v>
+        <v>105</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>357</v>
+        <v>106</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -6495,53 +6477,53 @@
         <v>79</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>354</v>
+        <v>107</v>
       </c>
       <c r="AG42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AH42" t="s" s="2">
         <v>90</v>
       </c>
-      <c r="AH42" t="s" s="2">
-        <v>81</v>
-      </c>
       <c r="AI42" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ42" t="s" s="2">
-        <v>358</v>
+        <v>79</v>
       </c>
       <c r="AK42" t="s" s="2">
-        <v>359</v>
+        <v>79</v>
       </c>
       <c r="AL42" t="s" s="2">
-        <v>360</v>
+        <v>108</v>
       </c>
       <c r="AM42" t="s" s="2">
-        <v>361</v>
+        <v>79</v>
       </c>
       <c r="AN42" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AO42" t="s" s="2">
-        <v>362</v>
+        <v>79</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
-        <v>79</v>
+        <v>110</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G43" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="H43" t="s" s="2">
         <v>79</v>
@@ -6553,15 +6535,17 @@
         <v>79</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>106</v>
-      </c>
-      <c r="N43" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="N43" t="s" s="2">
+        <v>114</v>
+      </c>
       <c r="O43" s="2"/>
       <c r="P43" t="s" s="2">
         <v>79</v>
@@ -6610,19 +6594,19 @@
         <v>79</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH43" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI43" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ43" t="s" s="2">
-        <v>79</v>
+        <v>119</v>
       </c>
       <c r="AK43" t="s" s="2">
         <v>79</v>
@@ -6642,14 +6626,14 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
-        <v>110</v>
+        <v>361</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
@@ -6662,24 +6646,26 @@
         <v>79</v>
       </c>
       <c r="I44" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="J44" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="K44" t="s" s="2">
         <v>111</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>112</v>
+        <v>362</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>113</v>
+        <v>363</v>
       </c>
       <c r="N44" t="s" s="2">
         <v>114</v>
       </c>
-      <c r="O44" s="2"/>
+      <c r="O44" t="s" s="2">
+        <v>207</v>
+      </c>
       <c r="P44" t="s" s="2">
         <v>79</v>
       </c>
@@ -6727,7 +6713,7 @@
         <v>79</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>118</v>
+        <v>364</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>80</v>
@@ -6745,7 +6731,7 @@
         <v>79</v>
       </c>
       <c r="AL44" t="s" s="2">
-        <v>108</v>
+        <v>193</v>
       </c>
       <c r="AM44" t="s" s="2">
         <v>79</v>
@@ -6766,7 +6752,7 @@
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
-        <v>366</v>
+        <v>79</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" t="s" s="2">
@@ -6779,26 +6765,24 @@
         <v>79</v>
       </c>
       <c r="I45" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="J45" t="s" s="2">
         <v>91</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>111</v>
+        <v>231</v>
       </c>
       <c r="L45" t="s" s="2">
+        <v>366</v>
+      </c>
+      <c r="M45" t="s" s="2">
         <v>367</v>
       </c>
-      <c r="M45" t="s" s="2">
+      <c r="N45" t="s" s="2">
         <v>368</v>
       </c>
-      <c r="N45" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="O45" t="s" s="2">
-        <v>212</v>
-      </c>
+      <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
         <v>79</v>
       </c>
@@ -6822,13 +6806,13 @@
         <v>79</v>
       </c>
       <c r="X45" t="s" s="2">
-        <v>79</v>
+        <v>152</v>
       </c>
       <c r="Y45" t="s" s="2">
-        <v>79</v>
+        <v>369</v>
       </c>
       <c r="Z45" t="s" s="2">
-        <v>79</v>
+        <v>370</v>
       </c>
       <c r="AA45" t="s" s="2">
         <v>79</v>
@@ -6846,7 +6830,7 @@
         <v>79</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>80</v>
@@ -6858,30 +6842,30 @@
         <v>79</v>
       </c>
       <c r="AJ45" t="s" s="2">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="AK45" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AL45" t="s" s="2">
-        <v>193</v>
+        <v>371</v>
       </c>
       <c r="AM45" t="s" s="2">
-        <v>79</v>
+        <v>108</v>
       </c>
       <c r="AN45" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AO45" t="s" s="2">
-        <v>79</v>
+        <v>372</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -6892,7 +6876,7 @@
         <v>80</v>
       </c>
       <c r="G46" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H46" t="s" s="2">
         <v>79</v>
@@ -6904,17 +6888,15 @@
         <v>91</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>236</v>
+        <v>374</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>372</v>
-      </c>
-      <c r="N46" t="s" s="2">
-        <v>373</v>
-      </c>
+        <v>376</v>
+      </c>
+      <c r="N46" s="2"/>
       <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
         <v>79</v>
@@ -6939,13 +6921,13 @@
         <v>79</v>
       </c>
       <c r="X46" t="s" s="2">
-        <v>152</v>
+        <v>79</v>
       </c>
       <c r="Y46" t="s" s="2">
-        <v>374</v>
+        <v>79</v>
       </c>
       <c r="Z46" t="s" s="2">
-        <v>375</v>
+        <v>79</v>
       </c>
       <c r="AA46" t="s" s="2">
         <v>79</v>
@@ -6963,13 +6945,13 @@
         <v>79</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH46" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="AI46" t="s" s="2">
         <v>79</v>
@@ -6981,24 +6963,24 @@
         <v>79</v>
       </c>
       <c r="AL46" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="AM46" t="s" s="2">
-        <v>108</v>
+        <v>378</v>
       </c>
       <c r="AN46" t="s" s="2">
-        <v>79</v>
+        <v>379</v>
       </c>
       <c r="AO46" t="s" s="2">
-        <v>377</v>
+        <v>380</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7021,13 +7003,13 @@
         <v>91</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>379</v>
+        <v>170</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="N47" s="2"/>
       <c r="O47" s="2"/>
@@ -7054,13 +7036,13 @@
         <v>79</v>
       </c>
       <c r="X47" t="s" s="2">
-        <v>79</v>
+        <v>222</v>
       </c>
       <c r="Y47" t="s" s="2">
-        <v>79</v>
+        <v>384</v>
       </c>
       <c r="Z47" t="s" s="2">
-        <v>79</v>
+        <v>385</v>
       </c>
       <c r="AA47" t="s" s="2">
         <v>79</v>
@@ -7078,7 +7060,7 @@
         <v>79</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>80</v>
@@ -7096,24 +7078,24 @@
         <v>79</v>
       </c>
       <c r="AL47" t="s" s="2">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="AM47" t="s" s="2">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="AN47" t="s" s="2">
-        <v>384</v>
+        <v>79</v>
       </c>
       <c r="AO47" t="s" s="2">
-        <v>385</v>
+        <v>79</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7121,7 +7103,7 @@
       </c>
       <c r="E48" s="2"/>
       <c r="F48" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G48" t="s" s="2">
         <v>90</v>
@@ -7139,10 +7121,10 @@
         <v>170</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
@@ -7169,13 +7151,13 @@
         <v>79</v>
       </c>
       <c r="X48" t="s" s="2">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="Y48" t="s" s="2">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="Z48" t="s" s="2">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="AA48" t="s" s="2">
         <v>79</v>
@@ -7193,10 +7175,10 @@
         <v>79</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="AG48" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="AH48" t="s" s="2">
         <v>90</v>
@@ -7211,24 +7193,24 @@
         <v>79</v>
       </c>
       <c r="AL48" t="s" s="2">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="AM48" t="s" s="2">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="AN48" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AO48" t="s" s="2">
-        <v>79</v>
+        <v>395</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -7236,7 +7218,7 @@
       </c>
       <c r="E49" s="2"/>
       <c r="F49" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G49" t="s" s="2">
         <v>90</v>
@@ -7248,16 +7230,16 @@
         <v>79</v>
       </c>
       <c r="J49" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>170</v>
+        <v>397</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>395</v>
+        <v>399</v>
       </c>
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
@@ -7284,34 +7266,34 @@
         <v>79</v>
       </c>
       <c r="X49" t="s" s="2">
-        <v>227</v>
+        <v>79</v>
       </c>
       <c r="Y49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Z49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AA49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AB49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AC49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF49" t="s" s="2">
         <v>396</v>
       </c>
-      <c r="Z49" t="s" s="2">
-        <v>397</v>
-      </c>
-      <c r="AA49" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB49" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC49" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD49" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE49" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF49" t="s" s="2">
-        <v>393</v>
-      </c>
       <c r="AG49" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="AH49" t="s" s="2">
         <v>90</v>
@@ -7326,24 +7308,24 @@
         <v>79</v>
       </c>
       <c r="AL49" t="s" s="2">
-        <v>398</v>
+        <v>108</v>
       </c>
       <c r="AM49" t="s" s="2">
-        <v>399</v>
+        <v>79</v>
       </c>
       <c r="AN49" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AO49" t="s" s="2">
-        <v>400</v>
+        <v>79</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -7354,7 +7336,7 @@
         <v>80</v>
       </c>
       <c r="G50" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="H50" t="s" s="2">
         <v>79</v>
@@ -7366,15 +7348,17 @@
         <v>79</v>
       </c>
       <c r="K50" t="s" s="2">
+        <v>397</v>
+      </c>
+      <c r="L50" t="s" s="2">
+        <v>401</v>
+      </c>
+      <c r="M50" t="s" s="2">
         <v>402</v>
       </c>
-      <c r="L50" t="s" s="2">
+      <c r="N50" t="s" s="2">
         <v>403</v>
       </c>
-      <c r="M50" t="s" s="2">
-        <v>404</v>
-      </c>
-      <c r="N50" s="2"/>
       <c r="O50" s="2"/>
       <c r="P50" t="s" s="2">
         <v>79</v>
@@ -7423,13 +7407,13 @@
         <v>79</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH50" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI50" t="s" s="2">
         <v>79</v>
@@ -7438,10 +7422,10 @@
         <v>102</v>
       </c>
       <c r="AK50" t="s" s="2">
-        <v>79</v>
+        <v>300</v>
       </c>
       <c r="AL50" t="s" s="2">
-        <v>108</v>
+        <v>404</v>
       </c>
       <c r="AM50" t="s" s="2">
         <v>79</v>
@@ -7450,124 +7434,7 @@
         <v>79</v>
       </c>
       <c r="AO50" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="s" s="2">
         <v>405</v>
-      </c>
-      <c r="B51" t="s" s="2">
-        <v>405</v>
-      </c>
-      <c r="C51" s="2"/>
-      <c r="D51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E51" s="2"/>
-      <c r="F51" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G51" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="K51" t="s" s="2">
-        <v>402</v>
-      </c>
-      <c r="L51" t="s" s="2">
-        <v>406</v>
-      </c>
-      <c r="M51" t="s" s="2">
-        <v>407</v>
-      </c>
-      <c r="N51" t="s" s="2">
-        <v>408</v>
-      </c>
-      <c r="O51" s="2"/>
-      <c r="P51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q51" s="2"/>
-      <c r="R51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF51" t="s" s="2">
-        <v>405</v>
-      </c>
-      <c r="AG51" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH51" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AJ51" t="s" s="2">
-        <v>102</v>
-      </c>
-      <c r="AK51" t="s" s="2">
-        <v>305</v>
-      </c>
-      <c r="AL51" t="s" s="2">
-        <v>409</v>
-      </c>
-      <c r="AM51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN51" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AO51" t="s" s="2">
-        <v>410</v>
       </c>
     </row>
   </sheetData>

</xml_diff>